<commit_message>
docs(report): update test report sheet generator and complete test execution report
- Updated generate-report.js to change the Unit Testing count to 41 and the total to 108

- Rebuilt GPP_Pharmacy_Test_Report_Detailed.xlsx with accurate test case counts

- Fully populated TEST_REPORT.md with final test execution metrics and details (108/108 PASS)
</commit_message>
<xml_diff>
--- a/GPP_Pharmacy_Test_Report_Detailed.xlsx
+++ b/GPP_Pharmacy_Test_Report_Detailed.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="638">
   <si>
     <t>BÁO CÁO KIỂM THỬ VÀ ĐẢM BẢO CHẤT LƯỢNG PHẦN MỀM</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Ngày kiểm thử:</t>
   </si>
   <si>
-    <t>4/6/2026</t>
+    <t>5/6/2026</t>
   </si>
   <si>
     <t>Mô tả:</t>
@@ -93,22 +93,25 @@
     <t>Kiểm thử Đơn vị (Unit Testing)</t>
   </si>
   <si>
-    <t>Jest</t>
+    <t>Jest / Node</t>
+  </si>
+  <si>
+    <t>41/41 Đạt</t>
+  </si>
+  <si>
+    <t>Kiểm thử Chịu tải (Load Testing)</t>
+  </si>
+  <si>
+    <t>k6</t>
   </si>
   <si>
     <t>2/2 Đạt</t>
   </si>
   <si>
-    <t>Kiểm thử Chịu tải (Load Testing)</t>
-  </si>
-  <si>
-    <t>k6</t>
-  </si>
-  <si>
     <t>TỔNG CỘNG</t>
   </si>
   <si>
-    <t>69/69 Đạt</t>
+    <t>108/108 Đạt</t>
   </si>
   <si>
     <t>XÁC THỰC &amp; PHÂN QUYỀN</t>
@@ -2753,7 +2756,7 @@
         <v>25</v>
       </c>
       <c r="D12" s="8">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>26</v>
@@ -2776,7 +2779,7 @@
         <v>2</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>20</v>
@@ -2787,16 +2790,16 @@
         <v>2</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D14" s="14">
-        <v>69</v>
+        <v>108</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>20</v>
@@ -2832,7 +2835,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2844,36 +2847,36 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -2882,41 +2885,41 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F5" s="18"/>
       <c r="G5" s="19"/>
@@ -2926,13 +2929,13 @@
       <c r="A6" s="17"/>
       <c r="B6" s="18"/>
       <c r="C6" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F6" s="18"/>
       <c r="G6" s="19"/>
@@ -2940,41 +2943,41 @@
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="18"/>
       <c r="C8" s="18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="18"/>
       <c r="G8" s="19"/>
@@ -2984,13 +2987,13 @@
       <c r="A9" s="17"/>
       <c r="B9" s="18"/>
       <c r="C9" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="18"/>
       <c r="G9" s="19"/>
@@ -2998,41 +3001,41 @@
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="18"/>
       <c r="C11" s="18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F11" s="18"/>
       <c r="G11" s="19"/>
@@ -3040,41 +3043,41 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="18"/>
       <c r="C13" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F13" s="18"/>
       <c r="G13" s="19"/>
@@ -3082,41 +3085,41 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
       <c r="B15" s="18"/>
       <c r="C15" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F15" s="18"/>
       <c r="G15" s="19"/>
@@ -3126,13 +3129,13 @@
       <c r="A16" s="17"/>
       <c r="B16" s="18"/>
       <c r="C16" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="18"/>
       <c r="G16" s="19"/>
@@ -3140,41 +3143,41 @@
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E17" s="18" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="18"/>
       <c r="C18" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="19"/>
@@ -3184,13 +3187,13 @@
       <c r="A19" s="17"/>
       <c r="B19" s="18"/>
       <c r="C19" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="19"/>
@@ -3200,13 +3203,13 @@
       <c r="A20" s="17"/>
       <c r="B20" s="18"/>
       <c r="C20" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F20" s="18"/>
       <c r="G20" s="19"/>
@@ -3214,41 +3217,41 @@
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E21" s="18" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
       <c r="B22" s="18"/>
       <c r="C22" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F22" s="18"/>
       <c r="G22" s="19"/>
@@ -3258,13 +3261,13 @@
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="19"/>
@@ -3274,13 +3277,13 @@
       <c r="A24" s="17"/>
       <c r="B24" s="18"/>
       <c r="C24" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F24" s="18"/>
       <c r="G24" s="19"/>
@@ -3288,41 +3291,41 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E25" s="18" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H25" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F26" s="18"/>
       <c r="G26" s="19"/>
@@ -3332,13 +3335,13 @@
       <c r="A27" s="17"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F27" s="18"/>
       <c r="G27" s="19"/>
@@ -3348,13 +3351,13 @@
       <c r="A28" s="17"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F28" s="18"/>
       <c r="G28" s="19"/>
@@ -3362,41 +3365,41 @@
     </row>
     <row r="29" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="17"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F30" s="18"/>
       <c r="G30" s="19"/>
@@ -3404,41 +3407,41 @@
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H31" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
       <c r="B32" s="18"/>
       <c r="C32" s="18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F32" s="18"/>
       <c r="G32" s="19"/>
@@ -3448,13 +3451,13 @@
       <c r="A33" s="17"/>
       <c r="B33" s="18"/>
       <c r="C33" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F33" s="18"/>
       <c r="G33" s="19"/>
@@ -3462,41 +3465,41 @@
     </row>
     <row r="34" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="18"/>
       <c r="C35" s="18" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="19"/>
@@ -3504,7 +3507,7 @@
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B36" s="21"/>
       <c r="C36" s="21"/>
@@ -3605,7 +3608,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -3617,36 +3620,36 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -3655,41 +3658,41 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F5" s="18"/>
       <c r="G5" s="19"/>
@@ -3697,41 +3700,41 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="18"/>
       <c r="C7" s="18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F7" s="18"/>
       <c r="G7" s="19"/>
@@ -3739,67 +3742,67 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="18"/>
       <c r="C10" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F10" s="18"/>
       <c r="G10" s="19"/>
@@ -3807,142 +3810,142 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="18"/>
       <c r="C16" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>2</v>
@@ -3953,41 +3956,41 @@
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="18"/>
       <c r="C18" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="19"/>
@@ -3997,13 +4000,13 @@
       <c r="A19" s="17"/>
       <c r="B19" s="18"/>
       <c r="C19" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="19"/>
@@ -4013,13 +4016,13 @@
       <c r="A20" s="17"/>
       <c r="B20" s="18"/>
       <c r="C20" s="18" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F20" s="18"/>
       <c r="G20" s="19"/>
@@ -4029,13 +4032,13 @@
       <c r="A21" s="17"/>
       <c r="B21" s="18"/>
       <c r="C21" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F21" s="18"/>
       <c r="G21" s="19"/>
@@ -4043,41 +4046,41 @@
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H22" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="19"/>
@@ -4087,13 +4090,13 @@
       <c r="A24" s="17"/>
       <c r="B24" s="18"/>
       <c r="C24" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F24" s="18"/>
       <c r="G24" s="19"/>
@@ -4101,41 +4104,41 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H25" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F26" s="18"/>
       <c r="G26" s="19"/>
@@ -4145,10 +4148,10 @@
       <c r="A27" s="17"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E27" s="18" t="s">
         <v>2</v>
@@ -4159,41 +4162,41 @@
     </row>
     <row r="28" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F29" s="18"/>
       <c r="G29" s="19"/>
@@ -4201,38 +4204,38 @@
     </row>
     <row r="30" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E31" s="18" t="s">
         <v>2</v>
@@ -4243,41 +4246,41 @@
     </row>
     <row r="32" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H32" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="17"/>
       <c r="B33" s="18"/>
       <c r="C33" s="18" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F33" s="18"/>
       <c r="G33" s="19"/>
@@ -4285,41 +4288,41 @@
     </row>
     <row r="34" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="18"/>
       <c r="C35" s="18" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="19"/>
@@ -4327,7 +4330,7 @@
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B36" s="23"/>
       <c r="C36" s="23"/>
@@ -4428,7 +4431,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -4440,36 +4443,36 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -4478,41 +4481,41 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F5" s="18"/>
       <c r="G5" s="19"/>
@@ -4520,93 +4523,93 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="18"/>
       <c r="C9" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F9" s="18"/>
       <c r="G9" s="19"/>
@@ -4614,41 +4617,41 @@
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="18"/>
       <c r="C11" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F11" s="18"/>
       <c r="G11" s="19"/>
@@ -4656,41 +4659,41 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="18"/>
       <c r="C13" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F13" s="18"/>
       <c r="G13" s="19"/>
@@ -4698,41 +4701,41 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
       <c r="B15" s="18"/>
       <c r="C15" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F15" s="18"/>
       <c r="G15" s="19"/>
@@ -4740,93 +4743,93 @@
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H16" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H18" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="17"/>
       <c r="B19" s="18"/>
       <c r="C19" s="18" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="19"/>
@@ -4834,41 +4837,41 @@
     </row>
     <row r="20" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="B21" s="18"/>
       <c r="C21" s="18" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F21" s="18"/>
       <c r="G21" s="19"/>
@@ -4878,13 +4881,13 @@
       <c r="A22" s="17"/>
       <c r="B22" s="18"/>
       <c r="C22" s="18" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F22" s="18"/>
       <c r="G22" s="19"/>
@@ -4894,13 +4897,13 @@
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="19"/>
@@ -4908,41 +4911,41 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H24" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F25" s="18"/>
       <c r="G25" s="19"/>
@@ -4952,13 +4955,13 @@
       <c r="A26" s="17"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F26" s="18"/>
       <c r="G26" s="19"/>
@@ -4968,13 +4971,13 @@
       <c r="A27" s="17"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F27" s="18"/>
       <c r="G27" s="19"/>
@@ -4982,41 +4985,41 @@
     </row>
     <row r="28" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F29" s="18"/>
       <c r="G29" s="19"/>
@@ -5026,13 +5029,13 @@
       <c r="A30" s="17"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F30" s="18"/>
       <c r="G30" s="19"/>
@@ -5040,41 +5043,41 @@
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H31" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
       <c r="B32" s="18"/>
       <c r="C32" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F32" s="18"/>
       <c r="G32" s="19"/>
@@ -5084,13 +5087,13 @@
       <c r="A33" s="17"/>
       <c r="B33" s="18"/>
       <c r="C33" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F33" s="18"/>
       <c r="G33" s="19"/>
@@ -5098,41 +5101,41 @@
     </row>
     <row r="34" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="18"/>
       <c r="C35" s="18" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="19"/>
@@ -5142,13 +5145,13 @@
       <c r="A36" s="17"/>
       <c r="B36" s="18"/>
       <c r="C36" s="18" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F36" s="18"/>
       <c r="G36" s="19"/>
@@ -5156,41 +5159,41 @@
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F37" s="18" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H37" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="17"/>
       <c r="B38" s="18"/>
       <c r="C38" s="18" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F38" s="18"/>
       <c r="G38" s="19"/>
@@ -5200,13 +5203,13 @@
       <c r="A39" s="17"/>
       <c r="B39" s="18"/>
       <c r="C39" s="18" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F39" s="18"/>
       <c r="G39" s="19"/>
@@ -5214,41 +5217,41 @@
     </row>
     <row r="40" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F40" s="18" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H40" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="17"/>
       <c r="B41" s="18"/>
       <c r="C41" s="18" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F41" s="18"/>
       <c r="G41" s="19"/>
@@ -5256,41 +5259,41 @@
     </row>
     <row r="42" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D42" s="18" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F42" s="18" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H42" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="17"/>
       <c r="B43" s="18"/>
       <c r="C43" s="18" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E43" s="18" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F43" s="18"/>
       <c r="G43" s="19"/>
@@ -5298,41 +5301,41 @@
     </row>
     <row r="44" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F44" s="18" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="17"/>
       <c r="B45" s="18"/>
       <c r="C45" s="18" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F45" s="18"/>
       <c r="G45" s="19"/>
@@ -5340,41 +5343,41 @@
     </row>
     <row r="46" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E46" s="18" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F46" s="18" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H46" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="17"/>
       <c r="B47" s="18"/>
       <c r="C47" s="18" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E47" s="18" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F47" s="18"/>
       <c r="G47" s="19"/>
@@ -5382,7 +5385,7 @@
     </row>
     <row r="48" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="25" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B48" s="25"/>
       <c r="C48" s="25"/>
@@ -5508,7 +5511,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -5520,36 +5523,36 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -5558,67 +5561,67 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="18"/>
       <c r="C6" s="18" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F6" s="18"/>
       <c r="G6" s="19"/>
@@ -5626,41 +5629,41 @@
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="18"/>
       <c r="C8" s="18" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F8" s="18"/>
       <c r="G8" s="19"/>
@@ -5668,93 +5671,93 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="18"/>
       <c r="C12" s="18" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F12" s="18"/>
       <c r="G12" s="19"/>
@@ -5762,93 +5765,93 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="18"/>
       <c r="C16" s="18" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F16" s="18"/>
       <c r="G16" s="19"/>
@@ -5856,41 +5859,41 @@
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="18"/>
       <c r="C18" s="18" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F18" s="18"/>
       <c r="G18" s="19"/>
@@ -5900,13 +5903,13 @@
       <c r="A19" s="17"/>
       <c r="B19" s="18"/>
       <c r="C19" s="18" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="19"/>
@@ -5916,13 +5919,13 @@
       <c r="A20" s="17"/>
       <c r="B20" s="18"/>
       <c r="C20" s="18" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F20" s="18"/>
       <c r="G20" s="19"/>
@@ -5930,41 +5933,41 @@
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
       <c r="B22" s="18"/>
       <c r="C22" s="18" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F22" s="18"/>
       <c r="G22" s="19"/>
@@ -5974,13 +5977,13 @@
       <c r="A23" s="17"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="19"/>
@@ -5988,38 +5991,38 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H24" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E25" s="18" t="s">
         <v>2</v>
@@ -6030,38 +6033,38 @@
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H26" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E27" s="18" t="s">
         <v>2</v>
@@ -6072,41 +6075,41 @@
     </row>
     <row r="28" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F29" s="18"/>
       <c r="G29" s="19"/>
@@ -6116,13 +6119,13 @@
       <c r="A30" s="17"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="F30" s="18"/>
       <c r="G30" s="19"/>
@@ -6132,13 +6135,13 @@
       <c r="A31" s="17"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F31" s="18"/>
       <c r="G31" s="19"/>
@@ -6146,41 +6149,41 @@
     </row>
     <row r="32" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H32" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="17"/>
       <c r="B33" s="18"/>
       <c r="C33" s="18" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="F33" s="18"/>
       <c r="G33" s="19"/>
@@ -6188,41 +6191,41 @@
     </row>
     <row r="34" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="18"/>
       <c r="C35" s="18" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="19"/>
@@ -6230,41 +6233,41 @@
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F36" s="18" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H36" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="17"/>
       <c r="B37" s="18"/>
       <c r="C37" s="18" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F37" s="18"/>
       <c r="G37" s="19"/>
@@ -6272,38 +6275,38 @@
     </row>
     <row r="38" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F38" s="18" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H38" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="17"/>
       <c r="B39" s="18"/>
       <c r="C39" s="18" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E39" s="18" t="s">
         <v>2</v>
@@ -6314,7 +6317,7 @@
     </row>
     <row r="40" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="27" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B40" s="27"/>
       <c r="C40" s="27"/>
@@ -6425,7 +6428,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
@@ -6437,36 +6440,36 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -6475,38 +6478,38 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>2</v>
@@ -6519,13 +6522,13 @@
       <c r="A6" s="17"/>
       <c r="B6" s="18"/>
       <c r="C6" s="18" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F6" s="18"/>
       <c r="G6" s="19"/>
@@ -6535,13 +6538,13 @@
       <c r="A7" s="17"/>
       <c r="B7" s="18"/>
       <c r="C7" s="18" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F7" s="18"/>
       <c r="G7" s="19"/>
@@ -6549,38 +6552,38 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="18"/>
       <c r="C9" s="18" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>2</v>
@@ -6593,13 +6596,13 @@
       <c r="A10" s="17"/>
       <c r="B10" s="18"/>
       <c r="C10" s="18" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="F10" s="18"/>
       <c r="G10" s="19"/>
@@ -6609,13 +6612,13 @@
       <c r="A11" s="17"/>
       <c r="B11" s="18"/>
       <c r="C11" s="18" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="F11" s="18"/>
       <c r="G11" s="19"/>
@@ -6623,41 +6626,41 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="18"/>
       <c r="C13" s="18" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F13" s="18"/>
       <c r="G13" s="19"/>
@@ -6667,13 +6670,13 @@
       <c r="A14" s="17"/>
       <c r="B14" s="18"/>
       <c r="C14" s="18" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F14" s="18"/>
       <c r="G14" s="19"/>
@@ -6681,41 +6684,41 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="18"/>
       <c r="C16" s="18" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F16" s="18"/>
       <c r="G16" s="19"/>
@@ -6725,13 +6728,13 @@
       <c r="A17" s="17"/>
       <c r="B17" s="18"/>
       <c r="C17" s="18" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F17" s="18"/>
       <c r="G17" s="19"/>
@@ -6739,7 +6742,7 @@
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B18" s="29"/>
       <c r="C18" s="29"/>

</xml_diff>